<commit_message>
Still 10 articles to go
</commit_message>
<xml_diff>
--- a/05_coding/atlas/Literature Review MDIMs – Code List.xlsx
+++ b/05_coding/atlas/Literature Review MDIMs – Code List.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="289">
   <si>
     <t>Code</t>
   </si>
@@ -2754,6 +2754,17 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
+      <t>Solution Interoperability Mechanism: Deep learning / AI</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF46AA00"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
       <t>Solution Interoperability Mechanism: Hybrid</t>
     </r>
   </si>
@@ -3092,6 +3103,17 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
+      <t>Solution Modelling type: EDI</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF46AA00"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
       <t>Solution Modelling type: Ontology</t>
     </r>
   </si>
@@ -3186,6 +3208,17 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
+      <t>Solution Modelling type: RosettaNet</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF46AA00"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
       <t>Solution Modelling type: SHACL</t>
     </r>
   </si>
@@ -3212,6 +3245,17 @@
 2. Pure XML Schema authored without UML lineage.
 Notes:
 Empirically thin, often present in figures rather than narrative text; retained for completeness because INSPIRE and the OSLO programme make extensive use of UML.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF46AA00"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Solution Modelling type: Vector Database</t>
+    </r>
   </si>
   <si>
     <r>
@@ -4261,8 +4305,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{c4982660-d5c4-4ea4-a21c-63a454417822}">
-  <dimension ref="A1:E147"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{e7ff6755-9d12-41ad-97f8-04e95bd17a8d}">
+  <dimension ref="A1:E151"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="80.42857142857143" customWidth="1"/>
@@ -5564,139 +5608,135 @@
       <c r="A105" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="B105" s="2" t="s">
-        <v>208</v>
-      </c>
+      <c r="B105" s="2"/>
       <c r="C105" s="2"/>
       <c r="D105" s="2"/>
-      <c r="E105" s="2" t="s">
-        <v>190</v>
-      </c>
+      <c r="E105" s="2"/>
     </row>
     <row r="106" spans="1:5" ht="14.25">
       <c r="A106" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B106" s="2" t="s">
         <v>209</v>
-      </c>
-      <c r="B106" s="2" t="s">
-        <v>210</v>
       </c>
       <c r="C106" s="2"/>
       <c r="D106" s="2"/>
-      <c r="E106" s="2"/>
+      <c r="E106" s="2" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="107" spans="1:5" ht="14.25">
       <c r="A107" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="B107" s="2" t="s">
         <v>211</v>
-      </c>
-      <c r="B107" s="2" t="s">
-        <v>212</v>
       </c>
       <c r="C107" s="2"/>
       <c r="D107" s="2"/>
-      <c r="E107" s="2" t="s">
-        <v>190</v>
-      </c>
+      <c r="E107" s="2"/>
     </row>
     <row r="108" spans="1:5" ht="14.25">
       <c r="A108" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="B108" s="2" t="s">
         <v>213</v>
-      </c>
-      <c r="B108" s="2" t="s">
-        <v>214</v>
       </c>
       <c r="C108" s="2"/>
       <c r="D108" s="2"/>
-      <c r="E108" s="2"/>
+      <c r="E108" s="2" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="109" spans="1:5" ht="14.25">
       <c r="A109" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="B109" s="2" t="s">
         <v>215</v>
-      </c>
-      <c r="B109" s="2" t="s">
-        <v>216</v>
       </c>
       <c r="C109" s="2"/>
       <c r="D109" s="2"/>
-      <c r="E109" s="2" t="s">
-        <v>190</v>
-      </c>
+      <c r="E109" s="2"/>
     </row>
     <row r="110" spans="1:5" ht="14.25">
       <c r="A110" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B110" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="B110" s="2"/>
       <c r="C110" s="2"/>
       <c r="D110" s="2"/>
-      <c r="E110" s="2"/>
+      <c r="E110" s="2" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="111" spans="1:5" ht="14.25">
       <c r="A111" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="B111" s="2" t="s">
-        <v>219</v>
-      </c>
+      <c r="B111" s="2"/>
       <c r="C111" s="2"/>
       <c r="D111" s="2"/>
-      <c r="E111" s="2" t="s">
-        <v>190</v>
-      </c>
+      <c r="E111" s="2"/>
     </row>
     <row r="112" spans="1:5" ht="14.25">
       <c r="A112" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="B112" s="2" t="s">
         <v>220</v>
-      </c>
-      <c r="B112" s="2" t="s">
-        <v>221</v>
       </c>
       <c r="C112" s="2"/>
       <c r="D112" s="2"/>
-      <c r="E112" s="2"/>
+      <c r="E112" s="2" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="113" spans="1:5" ht="14.25">
       <c r="A113" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B113" s="2" t="s">
         <v>222</v>
-      </c>
-      <c r="B113" s="2" t="s">
-        <v>223</v>
       </c>
       <c r="C113" s="2"/>
       <c r="D113" s="2"/>
-      <c r="E113" s="2" t="s">
-        <v>190</v>
-      </c>
+      <c r="E113" s="2"/>
     </row>
     <row r="114" spans="1:5" ht="14.25">
       <c r="A114" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B114" s="2" t="s">
         <v>224</v>
-      </c>
-      <c r="B114" s="2" t="s">
-        <v>225</v>
       </c>
       <c r="C114" s="2"/>
       <c r="D114" s="2"/>
-      <c r="E114" s="2"/>
+      <c r="E114" s="2" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="115" spans="1:5" ht="14.25">
       <c r="A115" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B115" s="2" t="s">
         <v>226</v>
-      </c>
-      <c r="B115" s="2" t="s">
-        <v>227</v>
       </c>
       <c r="C115" s="2"/>
       <c r="D115" s="2"/>
-      <c r="E115" s="2" t="s">
-        <v>190</v>
-      </c>
+      <c r="E115" s="2"/>
     </row>
     <row r="116" spans="1:5" ht="14.25">
       <c r="A116" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B116" s="2" t="s">
         <v>228</v>
-      </c>
-      <c r="B116" s="2" t="s">
-        <v>229</v>
       </c>
       <c r="C116" s="2"/>
       <c r="D116" s="2"/>
@@ -5706,21 +5746,23 @@
     </row>
     <row r="117" spans="1:5" ht="14.25">
       <c r="A117" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B117" s="2" t="s">
         <v>230</v>
-      </c>
-      <c r="B117" s="2" t="s">
-        <v>231</v>
       </c>
       <c r="C117" s="2"/>
       <c r="D117" s="2"/>
-      <c r="E117" s="2"/>
+      <c r="E117" s="2" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="118" spans="1:5" ht="14.25">
       <c r="A118" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="B118" s="2" t="s">
         <v>232</v>
-      </c>
-      <c r="B118" s="2" t="s">
-        <v>233</v>
       </c>
       <c r="C118" s="2"/>
       <c r="D118" s="2"/>
@@ -5728,29 +5770,31 @@
     </row>
     <row r="119" spans="1:5" ht="14.25">
       <c r="A119" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="B119" s="2" t="s">
-        <v>235</v>
-      </c>
+        <v>233</v>
+      </c>
+      <c r="B119" s="2"/>
       <c r="C119" s="2"/>
       <c r="D119" s="2"/>
       <c r="E119" s="2"/>
     </row>
     <row r="120" spans="1:5" ht="14.25">
       <c r="A120" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="B120" s="2"/>
+        <v>234</v>
+      </c>
+      <c r="B120" s="2" t="s">
+        <v>235</v>
+      </c>
       <c r="C120" s="2"/>
       <c r="D120" s="2"/>
       <c r="E120" s="2"/>
     </row>
     <row r="121" spans="1:5" ht="14.25">
       <c r="A121" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="B121" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="B121" s="2"/>
       <c r="C121" s="2"/>
       <c r="D121" s="2"/>
       <c r="E121" s="2"/>
@@ -5759,16 +5803,14 @@
       <c r="A122" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="B122" s="2" t="s">
-        <v>239</v>
-      </c>
+      <c r="B122" s="2"/>
       <c r="C122" s="2"/>
       <c r="D122" s="2"/>
       <c r="E122" s="2"/>
     </row>
     <row r="123" spans="1:5" ht="14.25">
       <c r="A123" s="2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B123" s="2"/>
       <c r="C123" s="2"/>
@@ -5777,10 +5819,10 @@
     </row>
     <row r="124" spans="1:5" ht="14.25">
       <c r="A124" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="B124" s="2" t="s">
         <v>241</v>
-      </c>
-      <c r="B124" s="2" t="s">
-        <v>242</v>
       </c>
       <c r="C124" s="2"/>
       <c r="D124" s="2"/>
@@ -5788,7 +5830,7 @@
     </row>
     <row r="125" spans="1:5" ht="14.25">
       <c r="A125" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B125" s="2"/>
       <c r="C125" s="2"/>
@@ -5797,7 +5839,7 @@
     </row>
     <row r="126" spans="1:5" ht="14.25">
       <c r="A126" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B126" s="2"/>
       <c r="C126" s="2"/>
@@ -5806,9 +5848,11 @@
     </row>
     <row r="127" spans="1:5" ht="14.25">
       <c r="A127" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="B127" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="B127" s="2"/>
       <c r="C127" s="2"/>
       <c r="D127" s="2"/>
       <c r="E127" s="2"/>
@@ -5817,60 +5861,44 @@
       <c r="A128" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="B128" s="2" t="s">
-        <v>247</v>
-      </c>
+      <c r="B128" s="2"/>
       <c r="C128" s="2"/>
       <c r="D128" s="2"/>
-      <c r="E128" s="2" t="s">
-        <v>190</v>
-      </c>
+      <c r="E128" s="2"/>
     </row>
     <row r="129" spans="1:5" ht="14.25">
       <c r="A129" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="B129" s="2" t="s">
-        <v>249</v>
-      </c>
+        <v>247</v>
+      </c>
+      <c r="B129" s="2"/>
       <c r="C129" s="2"/>
       <c r="D129" s="2"/>
-      <c r="E129" s="2" t="s">
-        <v>190</v>
-      </c>
+      <c r="E129" s="2"/>
     </row>
     <row r="130" spans="1:5" ht="14.25">
       <c r="A130" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="B130" s="2" t="s">
-        <v>251</v>
-      </c>
+        <v>248</v>
+      </c>
+      <c r="B130" s="2"/>
       <c r="C130" s="2"/>
       <c r="D130" s="2"/>
-      <c r="E130" s="2" t="s">
-        <v>190</v>
-      </c>
+      <c r="E130" s="2"/>
     </row>
     <row r="131" spans="1:5" ht="14.25">
       <c r="A131" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="B131" s="2" t="s">
-        <v>253</v>
-      </c>
+        <v>249</v>
+      </c>
+      <c r="B131" s="2"/>
       <c r="C131" s="2"/>
       <c r="D131" s="2"/>
-      <c r="E131" s="2" t="s">
-        <v>190</v>
-      </c>
+      <c r="E131" s="2"/>
     </row>
     <row r="132" spans="1:5" ht="14.25">
       <c r="A132" s="2" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="C132" s="2"/>
       <c r="D132" s="2"/>
@@ -5880,10 +5908,10 @@
     </row>
     <row r="133" spans="1:5" ht="14.25">
       <c r="A133" s="2" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="C133" s="2"/>
       <c r="D133" s="2"/>
@@ -5893,10 +5921,10 @@
     </row>
     <row r="134" spans="1:5" ht="14.25">
       <c r="A134" s="2" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="C134" s="2"/>
       <c r="D134" s="2"/>
@@ -5906,21 +5934,23 @@
     </row>
     <row r="135" spans="1:5" ht="14.25">
       <c r="A135" s="2" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="C135" s="2"/>
       <c r="D135" s="2"/>
-      <c r="E135" s="2"/>
+      <c r="E135" s="2" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="136" spans="1:5" ht="14.25">
       <c r="A136" s="2" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="C136" s="2"/>
       <c r="D136" s="2"/>
@@ -5930,10 +5960,10 @@
     </row>
     <row r="137" spans="1:5" ht="14.25">
       <c r="A137" s="2" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="C137" s="2"/>
       <c r="D137" s="2"/>
@@ -5943,21 +5973,23 @@
     </row>
     <row r="138" spans="1:5" ht="14.25">
       <c r="A138" s="2" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="C138" s="2"/>
       <c r="D138" s="2"/>
-      <c r="E138" s="2"/>
+      <c r="E138" s="2" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="139" spans="1:5" ht="14.25">
       <c r="A139" s="2" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="C139" s="2"/>
       <c r="D139" s="2"/>
@@ -5965,10 +5997,10 @@
     </row>
     <row r="140" spans="1:5" ht="14.25">
       <c r="A140" s="2" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="C140" s="2"/>
       <c r="D140" s="2"/>
@@ -5978,10 +6010,10 @@
     </row>
     <row r="141" spans="1:5" ht="14.25">
       <c r="A141" s="2" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="C141" s="2"/>
       <c r="D141" s="2"/>
@@ -5991,47 +6023,45 @@
     </row>
     <row r="142" spans="1:5" ht="14.25">
       <c r="A142" s="2" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="C142" s="2"/>
       <c r="D142" s="2"/>
-      <c r="E142" s="2" t="s">
-        <v>190</v>
-      </c>
+      <c r="E142" s="2"/>
     </row>
     <row r="143" spans="1:5" ht="14.25">
       <c r="A143" s="2" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="C143" s="2"/>
       <c r="D143" s="2"/>
-      <c r="E143" s="2" t="s">
-        <v>190</v>
-      </c>
+      <c r="E143" s="2"/>
     </row>
     <row r="144" spans="1:5" ht="14.25">
       <c r="A144" s="2" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="C144" s="2"/>
       <c r="D144" s="2"/>
-      <c r="E144" s="2"/>
+      <c r="E144" s="2" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="145" spans="1:5" ht="14.25">
       <c r="A145" s="2" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="C145" s="2"/>
       <c r="D145" s="2"/>
@@ -6041,10 +6071,10 @@
     </row>
     <row r="146" spans="1:5" ht="14.25">
       <c r="A146" s="2" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="C146" s="2"/>
       <c r="D146" s="2"/>
@@ -6054,12 +6084,62 @@
     </row>
     <row r="147" spans="1:5" ht="14.25">
       <c r="A147" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="B147" s="2"/>
+        <v>280</v>
+      </c>
+      <c r="B147" s="2" t="s">
+        <v>281</v>
+      </c>
       <c r="C147" s="2"/>
       <c r="D147" s="2"/>
-      <c r="E147" s="2"/>
+      <c r="E147" s="2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" ht="14.25">
+      <c r="A148" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="B148" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C148" s="2"/>
+      <c r="D148" s="2"/>
+      <c r="E148" s="2"/>
+    </row>
+    <row r="149" spans="1:5" ht="14.25">
+      <c r="A149" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="B149" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="C149" s="2"/>
+      <c r="D149" s="2"/>
+      <c r="E149" s="2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" ht="14.25">
+      <c r="A150" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="B150" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C150" s="2"/>
+      <c r="D150" s="2"/>
+      <c r="E150" s="2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" ht="14.25">
+      <c r="A151" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="B151" s="2"/>
+      <c r="C151" s="2"/>
+      <c r="D151" s="2"/>
+      <c r="E151" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>